<commit_message>
Sync v2_9_r2: CSVEncoding, csv NA/NULL text preservation, dependency bounds
- New required CSVEncoding column on ExternalFiles (utf-8, utf-8-sig,
  cp1251, cp1252); enforced by PreflightValidator and used by Importer
  to decode csv files. Existing workbooks must add the column.
- csv import no longer blanks literal text such as NULL, NA or N/A.
- Demo workbooks updated with the CSVEncoding column.
- pyproject.toml added; requirements.txt and requirements-dev.txt now
  carry version floors and a pandas <4 upper bound.
- FS v2_9_r2 added; FS v2_9_r1's v2_9_r0 row now reads "Initial version
  for public distribution."
- README.md: Python 3.14 requirement.

Full suite: 530 passed, 1 skipped (private-only real-Excel fixture).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/v2/demo/dimpolicy_ax.xlsx
+++ b/test_data/v2/demo/dimpolicy_ax.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="259">
   <si>
     <t xml:space="preserve">Item ID</t>
   </si>
@@ -747,6 +747,9 @@
     <t xml:space="preserve">CSVDelimiter</t>
   </si>
   <si>
+    <t xml:space="preserve">CSVEncoding</t>
+  </si>
+  <si>
     <t xml:space="preserve">test_data/v2/demo/items_ax.csv</t>
   </si>
   <si>
@@ -754,6 +757,9 @@
   </si>
   <si>
     <t xml:space="preserve">;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">utf-8</t>
   </si>
   <si>
     <t xml:space="preserve">test_data/v2/demo/whs_units.xlsx</t>
@@ -3867,7 +3873,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1048576"/>
+  <dimension ref="A1:H1048576"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.83"/>
@@ -3876,7 +3882,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="14.03"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3899,6 +3905,9 @@
         <v>239</v>
       </c>
       <c r="G1" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>160</v>
       </c>
     </row>
@@ -3907,18 +3916,21 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>163</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>146</v>
       </c>
     </row>
@@ -3927,19 +3939,20 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>202</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F3" s="3"/>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="3"/>
+      <c r="H3" s="3" t="s">
         <v>146</v>
       </c>
     </row>
@@ -3948,19 +3961,20 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>220</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F4" s="3"/>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="3"/>
+      <c r="H4" s="3" t="s">
         <v>146</v>
       </c>
     </row>
@@ -3969,7 +3983,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>223</v>
@@ -3978,10 +3992,11 @@
         <v>223</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F5" s="3"/>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="3"/>
+      <c r="H5" s="3" t="s">
         <v>146</v>
       </c>
     </row>
@@ -3990,18 +4005,21 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="G6" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>146</v>
       </c>
     </row>
@@ -4036,22 +4054,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>172</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G1" s="14" t="s">
         <v>160</v>
@@ -4065,11 +4083,11 @@
         <v>206</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D2" s="15"/>
       <c r="E2" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">

</xml_diff>